<commit_message>
Actualiza todo lo relacionado con el pipeline y la app de streamlit cargando todo lo nuevo desde la rama dev a día 26/02 23:00. - Añade nueva funcionalidad a la app - Añade los datasets de naturaleza y deporte - Perfecciona la documentación del uso de datos abiertos.
</commit_message>
<xml_diff>
--- a/etl-pipeline/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
+++ b/etl-pipeline/recursos/Tipos de actividades - TenerifeLifeScore.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="239">
   <si>
     <t>Sliders / Grupos</t>
   </si>
@@ -436,7 +436,7 @@
     <t>Mascotas</t>
   </si>
   <si>
-    <t>tienda de mascotas</t>
+    <t>mascotas</t>
   </si>
   <si>
     <t>Tiendas de mascotas</t>
@@ -448,13 +448,13 @@
     <t>Veterinarios</t>
   </si>
   <si>
-    <t>parque de mascotas</t>
+    <t>parque mascotas</t>
   </si>
   <si>
     <t>Parques de mascotas</t>
   </si>
   <si>
-    <t>playa de mascotas</t>
+    <t>playa mascotas</t>
   </si>
   <si>
     <t>Playas de mascotas</t>
@@ -691,7 +691,7 @@
     <t>parque deporte urbano</t>
   </si>
   <si>
-    <t>Ocio y picnic</t>
+    <t>Naturaleza</t>
   </si>
   <si>
     <t>Area recreativa</t>
@@ -703,16 +703,7 @@
     <t>Area de descanso</t>
   </si>
   <si>
-    <t>Educacion ambiental</t>
-  </si>
-  <si>
-    <t>Aula en la naturaleza</t>
-  </si>
-  <si>
-    <t>Aulas en la naturaleza</t>
-  </si>
-  <si>
-    <t>Paisaje y vistas</t>
+    <t>Aula en la Naturaleza</t>
   </si>
   <si>
     <t>Mirador</t>
@@ -752,7 +743,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d\-m"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -801,12 +792,7 @@
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
-      <name val="Droid Sans Mono"/>
-    </font>
-    <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
+      <name val="Oi"/>
     </font>
   </fonts>
   <fills count="4">
@@ -829,7 +815,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border/>
     <border>
       <left/>
@@ -863,16 +849,11 @@
       </top>
       <bottom/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -905,37 +886,16 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4402,7 +4362,7 @@
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="C45" s="18" t="s">
+      <c r="C45" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D45" s="6">
@@ -4419,10 +4379,10 @@
       <c r="B46" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="C46" s="19" t="s">
+      <c r="C46" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="D46" s="20">
+      <c r="D46" s="17">
         <v>8.0</v>
       </c>
       <c r="E46" s="17">
@@ -4433,7 +4393,7 @@
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="C47" s="21" t="s">
+      <c r="C47" s="18" t="s">
         <v>141</v>
       </c>
       <c r="D47" s="6">
@@ -4447,30 +4407,30 @@
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="C48" s="22" t="s">
+      <c r="C48" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="D48" s="23">
+      <c r="D48" s="6">
         <v>7.0</v>
       </c>
-      <c r="E48" s="23">
+      <c r="E48" s="6">
         <v>2.0</v>
       </c>
-      <c r="F48" s="23" t="s">
+      <c r="F48" s="6" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="C49" s="22" t="s">
+      <c r="C49" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="D49" s="23">
+      <c r="D49" s="6">
         <v>6.0</v>
       </c>
-      <c r="E49" s="23">
-        <v>3.0</v>
-      </c>
-      <c r="F49" s="23" t="s">
+      <c r="E49" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="F49" s="6" t="s">
         <v>146</v>
       </c>
     </row>
@@ -7102,13 +7062,13 @@
       <c r="B4" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="21">
         <v>10.0</v>
       </c>
-      <c r="E4" s="25">
+      <c r="E4" s="21">
         <v>4.0</v>
       </c>
       <c r="F4" s="7" t="s">
@@ -7116,13 +7076,13 @@
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="20" t="s">
         <v>211</v>
       </c>
-      <c r="D5" s="25">
+      <c r="D5" s="21">
         <v>10.0</v>
       </c>
-      <c r="E5" s="25">
+      <c r="E5" s="21">
         <v>1.0</v>
       </c>
       <c r="F5" s="7" t="s">
@@ -7130,238 +7090,238 @@
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="B22" s="24"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="B32" s="24"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="B34" s="24"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
+      <c r="B34" s="20"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="B35" s="24"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="B36" s="24"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="24"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="B40" s="24"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="24"/>
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="B41" s="24"/>
-      <c r="C41" s="24"/>
-      <c r="D41" s="24"/>
-      <c r="E41" s="24"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="B42" s="24"/>
-      <c r="C42" s="24"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="24"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="20"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="B43" s="24"/>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="B44" s="24"/>
-      <c r="C44" s="24"/>
-      <c r="D44" s="24"/>
-      <c r="E44" s="24"/>
+      <c r="B44" s="20"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
     </row>
     <row r="45" ht="15.75" customHeight="1"/>
     <row r="46" ht="15.75" customHeight="1"/>
@@ -8381,296 +8341,296 @@
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="20" t="s">
         <v>214</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="21">
         <v>10.0</v>
       </c>
-      <c r="E4" s="28">
+      <c r="E4" s="21">
         <v>5.0</v>
       </c>
-      <c r="F4" s="29" t="s">
+      <c r="F4" s="7" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="D5" s="28">
+      <c r="D5" s="21">
         <v>7.0</v>
       </c>
-      <c r="E5" s="25">
+      <c r="E5" s="21">
         <v>1.0</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F5" s="7" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="D6" s="27">
+      <c r="D6" s="20">
         <v>8.0</v>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="20">
         <v>1.0</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="6" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="D7" s="27">
+      <c r="D7" s="20">
         <v>10.0</v>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="20">
         <v>2.0</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="6" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="D8" s="27">
+      <c r="D8" s="20">
         <v>10.0</v>
       </c>
-      <c r="E8" s="27">
+      <c r="E8" s="20">
         <v>2.0</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="F8" s="6" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="B22" s="24"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="B32" s="24"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="B34" s="24"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
+      <c r="B34" s="20"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="B35" s="24"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="B36" s="24"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="24"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="B40" s="24"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="24"/>
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="B41" s="24"/>
-      <c r="C41" s="24"/>
-      <c r="D41" s="24"/>
-      <c r="E41" s="24"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="B42" s="24"/>
-      <c r="C42" s="24"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="24"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="20"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="B43" s="24"/>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="B44" s="24"/>
-      <c r="C44" s="24"/>
-      <c r="D44" s="24"/>
-      <c r="E44" s="24"/>
+      <c r="B44" s="20"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
     </row>
     <row r="45" ht="15.75" customHeight="1"/>
     <row r="46" ht="15.75" customHeight="1"/>
@@ -9691,334 +9651,328 @@
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="21">
         <v>10.0</v>
       </c>
-      <c r="E4" s="28">
+      <c r="E4" s="21">
         <v>1.0</v>
       </c>
-      <c r="F4" s="29" t="s">
+      <c r="F4" s="7" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="20" t="s">
         <v>227</v>
       </c>
-      <c r="D5" s="27">
+      <c r="D5" s="20">
         <v>8.0</v>
       </c>
-      <c r="E5" s="27">
+      <c r="E5" s="20">
         <v>1.0</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F5" s="7" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="B6" s="27" t="s">
+      <c r="C6" s="20" t="s">
         <v>228</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="D6" s="20">
+        <v>5.0</v>
+      </c>
+      <c r="E6" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="C7" s="20" t="s">
         <v>229</v>
       </c>
-      <c r="D6" s="27">
-        <v>5.0</v>
-      </c>
-      <c r="E6" s="27">
+      <c r="D7" s="20">
+        <v>10.0</v>
+      </c>
+      <c r="E7" s="22">
         <v>1.0</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F7" s="6" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="B7" s="27" t="s">
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="C8" s="20" t="s">
         <v>231</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="D8" s="20">
+        <v>7.0</v>
+      </c>
+      <c r="E8" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="D7" s="27">
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="B9" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="D9" s="20">
         <v>8.0</v>
       </c>
-      <c r="E7" s="27">
+      <c r="E9" s="20">
         <v>2.0</v>
       </c>
-      <c r="F7" s="23" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="8" ht="15.75" customHeight="1">
-      <c r="C8" s="27" t="s">
-        <v>234</v>
-      </c>
-      <c r="D8" s="27">
-        <v>5.0</v>
-      </c>
-      <c r="E8" s="27">
+      <c r="F9" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="C10" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="D10" s="20">
+        <v>8.0</v>
+      </c>
+      <c r="E10" s="20">
+        <v>2.0</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="C11" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="D11" s="20">
+        <v>10.0</v>
+      </c>
+      <c r="E11" s="20">
         <v>1.0</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="F11" s="6" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1">
-      <c r="B9" s="27" t="s">
-        <v>236</v>
-      </c>
-      <c r="C9" s="27" t="s">
-        <v>237</v>
-      </c>
-      <c r="D9" s="27">
-        <v>7.0</v>
-      </c>
-      <c r="E9" s="27">
-        <v>2.0</v>
-      </c>
-      <c r="F9" s="23" t="s">
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="C12" s="20" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="10" ht="15.75" customHeight="1">
-      <c r="C10" s="27" t="s">
-        <v>239</v>
-      </c>
-      <c r="D10" s="27">
-        <v>7.0</v>
-      </c>
-      <c r="E10" s="27">
-        <v>2.0</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="C11" s="27" t="s">
-        <v>240</v>
-      </c>
-      <c r="D11" s="27">
-        <v>5.0</v>
-      </c>
-      <c r="E11" s="27">
+      <c r="D12" s="20">
+        <v>8.0</v>
+      </c>
+      <c r="E12" s="20">
         <v>1.0</v>
       </c>
-      <c r="F11" s="23" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="12" ht="15.75" customHeight="1">
-      <c r="C12" s="27" t="s">
-        <v>241</v>
-      </c>
-      <c r="D12" s="27">
-        <v>6.0</v>
-      </c>
-      <c r="E12" s="27">
-        <v>1.0</v>
-      </c>
-      <c r="F12" s="23" t="s">
-        <v>238</v>
+      <c r="F12" s="6" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="B22" s="24"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="B32" s="24"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="B34" s="24"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
+      <c r="B34" s="20"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="B35" s="24"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="B36" s="24"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="24"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="B40" s="24"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="24"/>
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="B41" s="24"/>
-      <c r="C41" s="24"/>
-      <c r="D41" s="24"/>
-      <c r="E41" s="24"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="B42" s="24"/>
-      <c r="C42" s="24"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="24"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="20"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="B43" s="24"/>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="B44" s="24"/>
-      <c r="C44" s="24"/>
-      <c r="D44" s="24"/>
-      <c r="E44" s="24"/>
+      <c r="B44" s="20"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
     </row>
     <row r="45" ht="15.75" customHeight="1"/>
     <row r="46" ht="15.75" customHeight="1"/>
@@ -10977,9 +10931,8 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B7:B8"/>
+  <mergeCells count="2">
+    <mergeCell ref="B4:B8"/>
     <mergeCell ref="B9:B12"/>
   </mergeCells>
   <printOptions/>

</xml_diff>